<commit_message>
patient registration update code commited by sree
</commit_message>
<xml_diff>
--- a/src/test/resources/ExcelData/Exceldata.xlsx
+++ b/src/test/resources/ExcelData/Exceldata.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Eclipse Workspace\SvcProject\src\test\resources\ExcelData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Git Projects\SvcProject\src\test\resources\ExcelData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5861F2B-FC9A-4F04-97CF-CFE78BFF25FC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C3B5C40-AA49-4969-9632-2A5DEFF408EF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" firstSheet="34" activeTab="39" xr2:uid="{933DE942-FB34-432E-983A-800C465E3B57}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" firstSheet="10" activeTab="13" xr2:uid="{933DE942-FB34-432E-983A-800C465E3B57}"/>
   </bookViews>
   <sheets>
     <sheet name="signupscenarios1" sheetId="5" r:id="rId1"/>
@@ -25,34 +25,38 @@
     <sheet name="forgotpasswordscenario4" sheetId="30" r:id="rId10"/>
     <sheet name="patientprofile" sheetId="4" r:id="rId11"/>
     <sheet name="patientregistration" sheetId="9" r:id="rId12"/>
-    <sheet name="bookappointment" sheetId="10" r:id="rId13"/>
-    <sheet name="doctorregistration" sheetId="11" r:id="rId14"/>
-    <sheet name="doctorprofile" sheetId="40" r:id="rId15"/>
-    <sheet name="staffregistration" sheetId="12" r:id="rId16"/>
-    <sheet name="svcregistration" sheetId="13" r:id="rId17"/>
-    <sheet name="specialization" sheetId="14" r:id="rId18"/>
-    <sheet name="commandcenter1" sheetId="15" r:id="rId19"/>
-    <sheet name="commandcenter2" sheetId="33" r:id="rId20"/>
-    <sheet name="slotconfiguration" sheetId="16" r:id="rId21"/>
-    <sheet name="assetmaster1" sheetId="17" r:id="rId22"/>
-    <sheet name="assetmaster2" sheetId="35" r:id="rId23"/>
-    <sheet name="assetdetails1" sheetId="18" r:id="rId24"/>
-    <sheet name="assetdetails2" sheetId="36" r:id="rId25"/>
-    <sheet name="assetmapping1" sheetId="19" r:id="rId26"/>
-    <sheet name="assetmapping2" sheetId="37" r:id="rId27"/>
-    <sheet name="devicestatus1" sheetId="22" r:id="rId28"/>
-    <sheet name="devicestatus2" sheetId="38" r:id="rId29"/>
-    <sheet name="releasenote" sheetId="23" r:id="rId30"/>
-    <sheet name="raiseticket" sheetId="28" r:id="rId31"/>
-    <sheet name="myappointments" sheetId="32" r:id="rId32"/>
-    <sheet name="leave" sheetId="34" r:id="rId33"/>
-    <sheet name="notificationconfiguration" sheetId="39" r:id="rId34"/>
-    <sheet name="bulkcancellation" sheetId="41" r:id="rId35"/>
-    <sheet name="usermanagement" sheetId="42" r:id="rId36"/>
-    <sheet name="appointmentstatuschange" sheetId="43" r:id="rId37"/>
-    <sheet name="holidaycalendar" sheetId="44" r:id="rId38"/>
-    <sheet name="holidaycalendarstatus" sheetId="45" r:id="rId39"/>
-    <sheet name="holidaycalendaredit" sheetId="46" r:id="rId40"/>
+    <sheet name="patientregistrationdelete" sheetId="47" r:id="rId13"/>
+    <sheet name="patientregistrationdeactivate" sheetId="48" r:id="rId14"/>
+    <sheet name="patientregistrationupdate" sheetId="49" r:id="rId15"/>
+    <sheet name="patientregistrationview" sheetId="50" r:id="rId16"/>
+    <sheet name="bookappointment" sheetId="10" r:id="rId17"/>
+    <sheet name="doctorregistration" sheetId="11" r:id="rId18"/>
+    <sheet name="doctorprofile" sheetId="40" r:id="rId19"/>
+    <sheet name="staffregistration" sheetId="12" r:id="rId20"/>
+    <sheet name="svcregistration" sheetId="13" r:id="rId21"/>
+    <sheet name="specialization" sheetId="14" r:id="rId22"/>
+    <sheet name="commandcenter1" sheetId="15" r:id="rId23"/>
+    <sheet name="commandcenter2" sheetId="33" r:id="rId24"/>
+    <sheet name="slotconfiguration" sheetId="16" r:id="rId25"/>
+    <sheet name="assetmaster1" sheetId="17" r:id="rId26"/>
+    <sheet name="assetmaster2" sheetId="35" r:id="rId27"/>
+    <sheet name="assetdetails1" sheetId="18" r:id="rId28"/>
+    <sheet name="assetdetails2" sheetId="36" r:id="rId29"/>
+    <sheet name="assetmapping1" sheetId="19" r:id="rId30"/>
+    <sheet name="assetmapping2" sheetId="37" r:id="rId31"/>
+    <sheet name="devicestatus1" sheetId="22" r:id="rId32"/>
+    <sheet name="devicestatus2" sheetId="38" r:id="rId33"/>
+    <sheet name="releasenote" sheetId="23" r:id="rId34"/>
+    <sheet name="raiseticket" sheetId="28" r:id="rId35"/>
+    <sheet name="myappointments" sheetId="32" r:id="rId36"/>
+    <sheet name="leave" sheetId="34" r:id="rId37"/>
+    <sheet name="notificationconfiguration" sheetId="39" r:id="rId38"/>
+    <sheet name="bulkcancellation" sheetId="41" r:id="rId39"/>
+    <sheet name="usermanagement" sheetId="42" r:id="rId40"/>
+    <sheet name="appointmentstatuschange" sheetId="43" r:id="rId41"/>
+    <sheet name="holidaycalendar" sheetId="44" r:id="rId42"/>
+    <sheet name="holidaycalendarstatus" sheetId="45" r:id="rId43"/>
+    <sheet name="holidaycalendaredit" sheetId="46" r:id="rId44"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -64,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="376">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="390">
   <si>
     <t>username</t>
   </si>
@@ -1192,6 +1196,48 @@
   </si>
   <si>
     <t>Details Updated Successfully</t>
+  </si>
+  <si>
+    <t>DeleteAccountSearch</t>
+  </si>
+  <si>
+    <t>DeleteReason</t>
+  </si>
+  <si>
+    <t>8984498911</t>
+  </si>
+  <si>
+    <t>account delete</t>
+  </si>
+  <si>
+    <t>Account Deleted Successfully</t>
+  </si>
+  <si>
+    <t>AccountStatusSearch</t>
+  </si>
+  <si>
+    <t>DeactivateReason</t>
+  </si>
+  <si>
+    <t>7585469852</t>
+  </si>
+  <si>
+    <t>account deactivate</t>
+  </si>
+  <si>
+    <t>Patient - Mani Status Deactivated Successfully</t>
+  </si>
+  <si>
+    <t>EditSearch</t>
+  </si>
+  <si>
+    <t>Mani</t>
+  </si>
+  <si>
+    <t>ViewPatientSearch</t>
+  </si>
+  <si>
+    <t>7019619728</t>
   </si>
 </sst>
 </file>
@@ -2146,6 +2192,273 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D9CD3B3-9773-4EAB-BB74-06FFB1B22BA5}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" customWidth="1"/>
+    <col min="3" max="3" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>380</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2E62DAE-CA49-42FD-96AD-3646FEE5D187}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="42.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>385</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5ADEEAC-98DF-4835-9AA7-239FF4915CDA}">
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.28515625" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="33.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J1" t="s">
+        <v>45</v>
+      </c>
+      <c r="K1" t="s">
+        <v>46</v>
+      </c>
+      <c r="L1" t="s">
+        <v>47</v>
+      </c>
+      <c r="M1" t="s">
+        <v>246</v>
+      </c>
+      <c r="N1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2">
+        <v>7585469852</v>
+      </c>
+      <c r="K2">
+        <v>789123</v>
+      </c>
+      <c r="L2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M2" t="s">
+        <v>7</v>
+      </c>
+      <c r="N2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90B41094-CCCA-4C27-B328-C00C93A59B3E}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>389</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{245E0D39-D87F-4901-88CE-2EF066E1AE03}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2205,7 +2518,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7664799-BC46-4D3C-A5A1-CA40092AC2EF}">
   <dimension ref="A1:W2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2375,7 +2688,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59334133-C851-4E3B-8114-DBAC71D9F67C}">
   <dimension ref="A1:W2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2549,7 +2862,112 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{473E6D34-553A-4AD5-8C34-F30C656A6E7D}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.5703125" customWidth="1"/>
+    <col min="3" max="3" width="24.28515625" customWidth="1"/>
+    <col min="4" max="4" width="19.7109375" customWidth="1"/>
+    <col min="5" max="5" width="18.85546875" customWidth="1"/>
+    <col min="6" max="6" width="16.85546875" customWidth="1"/>
+    <col min="7" max="7" width="20.7109375" customWidth="1"/>
+    <col min="8" max="8" width="52.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>222</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{3312D515-F9FC-4C8C-A15F-749EE2FC7DD3}"/>
+    <hyperlink ref="D2" r:id="rId2" xr:uid="{95E53151-C3EA-427A-9B71-CB539C70940C}"/>
+    <hyperlink ref="C2" r:id="rId3" xr:uid="{BA710F4C-2DF9-4D87-8615-4E59B1A749C4}"/>
+    <hyperlink ref="E3" r:id="rId4" xr:uid="{54063B6B-A562-434C-A56D-DC7316709154}"/>
+    <hyperlink ref="D3" r:id="rId5" xr:uid="{0D273ABB-3D6F-4D1C-AB2E-A022B2FEC55E}"/>
+    <hyperlink ref="C3" r:id="rId6" xr:uid="{2083227D-79A3-44F0-98A6-FEFA591548F2}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2742953A-6D4D-4EE2-9C49-7917115B70D9}">
   <dimension ref="A1:W2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2727,7 +3145,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2FBCB0B-23F9-4860-8E3B-088250F105DD}">
   <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2841,7 +3259,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC313557-DBBA-4BB7-8126-A5BAC112B30A}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2939,7 +3357,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FB66439-7599-4005-A3F9-C47260664CD0}">
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3025,112 +3443,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{473E6D34-553A-4AD5-8C34-F30C656A6E7D}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="17.5703125" customWidth="1"/>
-    <col min="3" max="3" width="24.28515625" customWidth="1"/>
-    <col min="4" max="4" width="19.7109375" customWidth="1"/>
-    <col min="5" max="5" width="18.85546875" customWidth="1"/>
-    <col min="6" max="6" width="16.85546875" customWidth="1"/>
-    <col min="7" max="7" width="20.7109375" customWidth="1"/>
-    <col min="8" max="8" width="52.28515625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>222</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{3312D515-F9FC-4C8C-A15F-749EE2FC7DD3}"/>
-    <hyperlink ref="D2" r:id="rId2" xr:uid="{95E53151-C3EA-427A-9B71-CB539C70940C}"/>
-    <hyperlink ref="C2" r:id="rId3" xr:uid="{BA710F4C-2DF9-4D87-8615-4E59B1A749C4}"/>
-    <hyperlink ref="E3" r:id="rId4" xr:uid="{54063B6B-A562-434C-A56D-DC7316709154}"/>
-    <hyperlink ref="D3" r:id="rId5" xr:uid="{0D273ABB-3D6F-4D1C-AB2E-A022B2FEC55E}"/>
-    <hyperlink ref="C3" r:id="rId6" xr:uid="{2083227D-79A3-44F0-98A6-FEFA591548F2}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B49201DF-AA3E-41D0-BDA1-2299C31D0A4D}">
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3248,7 +3561,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40198505-B0DB-445A-B9CD-C4A358A7E367}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3305,7 +3618,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DFC1660-BBA4-4CFE-9D55-02214C348F4D}">
   <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3411,7 +3724,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90E994E8-C426-4AC4-A6CC-4C90E97C5A80}">
   <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3516,7 +3829,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F252328-6F51-44F6-B5E4-419C96527A4F}">
   <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3608,7 +3921,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6824B24B-16BA-4296-9D8E-6D77EAD5AB2C}">
   <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3701,223 +4014,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E49E0CC5-691C-40D2-BBBF-7332FA3007D6}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="14.42578125" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" customWidth="1"/>
-    <col min="3" max="3" width="24.140625" customWidth="1"/>
-    <col min="4" max="4" width="19.7109375" customWidth="1"/>
-    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="32.42578125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>338</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34F0824B-030E-47F6-A149-14317A06E7D4}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="32.42578125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>339</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3D0D13A-6A50-4D0F-B248-9DB6055A3A3A}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="15.5703125" customWidth="1"/>
-    <col min="2" max="2" width="17.42578125" customWidth="1"/>
-    <col min="3" max="3" width="61.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.28515625" customWidth="1"/>
-    <col min="5" max="5" width="37.7109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>342</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55EEE92C-EAEE-4186-ADEB-C3C60E4FCBD9}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="61.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="37.7109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>343</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{691B9017-0EEA-462A-A81D-4A9AC1615FEC}">
   <dimension ref="A1:D5"/>
@@ -4014,6 +4110,223 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E49E0CC5-691C-40D2-BBBF-7332FA3007D6}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.42578125" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" customWidth="1"/>
+    <col min="3" max="3" width="24.140625" customWidth="1"/>
+    <col min="4" max="4" width="19.7109375" customWidth="1"/>
+    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="32.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>338</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34F0824B-030E-47F6-A149-14317A06E7D4}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="32.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>339</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3D0D13A-6A50-4D0F-B248-9DB6055A3A3A}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.5703125" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" customWidth="1"/>
+    <col min="3" max="3" width="61.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.28515625" customWidth="1"/>
+    <col min="5" max="5" width="37.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>342</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55EEE92C-EAEE-4186-ADEB-C3C60E4FCBD9}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="37.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>343</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D99E86F1-FC1A-4C38-99D1-24F05E83496F}">
   <dimension ref="A1:P2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4141,7 +4454,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1376A961-1EAA-4397-8324-4DF710640D4C}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4199,7 +4512,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2495EE04-10E6-4E21-827B-FEDABF50D1ED}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4243,7 +4556,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E450965-A916-4D42-A891-1FBD5E746FB0}">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4322,7 +4635,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6B2F062-027B-43DA-BE0E-8C9D48A807AD}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4388,7 +4701,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9F72FB8-0EC3-417C-A79A-6BBD2A58D80D}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4452,271 +4765,6 @@
       </c>
       <c r="H2" s="1" t="s">
         <v>356</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C198979-6544-4CF5-A2FF-2A2620159074}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="14.5703125" customWidth="1"/>
-    <col min="2" max="2" width="10.28515625" customWidth="1"/>
-    <col min="3" max="3" width="33.140625" customWidth="1"/>
-    <col min="4" max="4" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.7109375" customWidth="1"/>
-    <col min="7" max="7" width="42.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="26" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>360</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>361</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>363</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>362</v>
-      </c>
-      <c r="H2" s="1"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="H3" s="1"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD3B6EFE-20F0-456E-8799-288CD86E6A3B}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="15.28515625" customWidth="1"/>
-    <col min="2" max="2" width="11.140625" customWidth="1"/>
-    <col min="3" max="3" width="32.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.85546875" customWidth="1"/>
-    <col min="6" max="6" width="20.28515625" customWidth="1"/>
-    <col min="7" max="7" width="22.42578125" customWidth="1"/>
-    <col min="8" max="8" width="50.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>340</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>365</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>325</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>366</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>367</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>363</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>364</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D450D9BB-F0D7-4040-9342-7F8A27F6754E}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="14.7109375" customWidth="1"/>
-    <col min="2" max="2" width="11.85546875" customWidth="1"/>
-    <col min="3" max="3" width="24.140625" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" customWidth="1"/>
-    <col min="5" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="50.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>368</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>369</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>372</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>370</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>371</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE7FDDFB-2BBA-469F-83B0-A4213156BAA4}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="13.28515625" customWidth="1"/>
-    <col min="2" max="2" width="11.7109375" customWidth="1"/>
-    <col min="3" max="3" width="17.85546875" customWidth="1"/>
-    <col min="4" max="4" width="19.28515625" customWidth="1"/>
-    <col min="5" max="5" width="20" customWidth="1"/>
-    <col min="6" max="6" width="26" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>373</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>325</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>372</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>370</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>374</v>
       </c>
     </row>
   </sheetData>
@@ -4782,6 +4830,271 @@
 </file>
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C198979-6544-4CF5-A2FF-2A2620159074}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.5703125" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" customWidth="1"/>
+    <col min="3" max="3" width="33.140625" customWidth="1"/>
+    <col min="4" max="4" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.7109375" customWidth="1"/>
+    <col min="7" max="7" width="42.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="H2" s="1"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="H3" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD3B6EFE-20F0-456E-8799-288CD86E6A3B}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.28515625" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" customWidth="1"/>
+    <col min="3" max="3" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.85546875" customWidth="1"/>
+    <col min="6" max="6" width="20.28515625" customWidth="1"/>
+    <col min="7" max="7" width="22.42578125" customWidth="1"/>
+    <col min="8" max="8" width="50.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>364</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D450D9BB-F0D7-4040-9342-7F8A27F6754E}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" customWidth="1"/>
+    <col min="3" max="3" width="24.140625" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="6" max="6" width="50.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>371</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE7FDDFB-2BBA-469F-83B0-A4213156BAA4}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.28515625" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" customWidth="1"/>
+    <col min="4" max="4" width="19.28515625" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="26" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>374</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{626522D9-2FFC-4159-9115-CB90B0A3A58D}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
signinvia otp updated code
</commit_message>
<xml_diff>
--- a/src/test/resources/ExcelData/Exceldata.xlsx
+++ b/src/test/resources/ExcelData/Exceldata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Git Projects\SvcProject\src\test\resources\ExcelData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37F6DA60-2337-4CDC-A1FF-9C84FCC472D2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{459EEAAB-B96B-4581-88D9-FA7130860174}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{933DE942-FB34-432E-983A-800C465E3B57}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" activeTab="4" xr2:uid="{933DE942-FB34-432E-983A-800C465E3B57}"/>
   </bookViews>
   <sheets>
     <sheet name="signupscenarios1" sheetId="5" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="389">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="390">
   <si>
     <t>username</t>
   </si>
@@ -1235,6 +1235,9 @@
   </si>
   <si>
     <t>8496345869</t>
+  </si>
+  <si>
+    <t>789129</t>
   </si>
 </sst>
 </file>
@@ -4811,7 +4814,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>11</v>
+        <v>389</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>8</v>

</xml_diff>

<commit_message>
change password update code and signinvia otp updated code
</commit_message>
<xml_diff>
--- a/src/test/resources/ExcelData/Exceldata.xlsx
+++ b/src/test/resources/ExcelData/Exceldata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Git Projects\SvcProject\src\test\resources\ExcelData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{459EEAAB-B96B-4581-88D9-FA7130860174}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4747744C-6093-433E-892F-46A87B155B6B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" activeTab="4" xr2:uid="{933DE942-FB34-432E-983A-800C465E3B57}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" activeTab="5" xr2:uid="{933DE942-FB34-432E-983A-800C465E3B57}"/>
   </bookViews>
   <sheets>
     <sheet name="signupscenarios1" sheetId="5" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="391">
   <si>
     <t>username</t>
   </si>
@@ -1238,6 +1238,9 @@
   </si>
   <si>
     <t>789129</t>
+  </si>
+  <si>
+    <t>Idea@123456</t>
   </si>
 </sst>
 </file>
@@ -5216,7 +5219,7 @@
         <v>37</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>89</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>34</v>
@@ -5238,8 +5241,8 @@
       <c r="A2" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>6</v>
+      <c r="B2" s="4" t="s">
+        <v>4</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>2</v>
@@ -5261,8 +5264,8 @@
       <c r="A3" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>6</v>
+      <c r="B3" s="4" t="s">
+        <v>4</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>6</v>
@@ -5284,8 +5287,8 @@
       <c r="A4" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>6</v>
+      <c r="B4" s="4" t="s">
+        <v>4</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>6</v>
@@ -5307,17 +5310,17 @@
       <c r="A5" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>6</v>
+      <c r="B5" s="4" t="s">
+        <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>2</v>
+        <v>390</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>2</v>
+        <v>390</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>7</v>
@@ -5331,22 +5334,18 @@
     <hyperlink ref="C2" r:id="rId1" xr:uid="{BA503714-DAF0-4123-AD4F-1C2191A846EB}"/>
     <hyperlink ref="D2" r:id="rId2" xr:uid="{854911C0-1041-4937-95C6-9B9863CC2C68}"/>
     <hyperlink ref="E2" r:id="rId3" xr:uid="{C607298D-AD77-4561-9DA9-6ED97D50F9AA}"/>
-    <hyperlink ref="B2" r:id="rId4" xr:uid="{348DAE75-624A-4B03-93BC-BA29DC672150}"/>
-    <hyperlink ref="C3" r:id="rId5" xr:uid="{548807EE-69C0-4A4D-8A04-AF2D97456A13}"/>
-    <hyperlink ref="D3" r:id="rId6" xr:uid="{5ECCA65F-D672-4C9C-8475-481CB035711B}"/>
-    <hyperlink ref="E3" r:id="rId7" xr:uid="{9CDE25A8-7826-4B6A-9CD2-DA248C33C664}"/>
-    <hyperlink ref="B3" r:id="rId8" xr:uid="{F0011DF8-E727-4E48-9CF6-21B5013F6C25}"/>
-    <hyperlink ref="C4" r:id="rId9" xr:uid="{4834B8AE-D2F2-46BB-B1FB-2917FB614179}"/>
-    <hyperlink ref="D4" r:id="rId10" xr:uid="{42D7F317-7486-4C56-8E8B-67291A0DFEBB}"/>
-    <hyperlink ref="E4" r:id="rId11" xr:uid="{3F8C1CEF-9B8C-42CD-8EA8-5A606E73DF96}"/>
-    <hyperlink ref="B4" r:id="rId12" xr:uid="{DDBDA5DF-883F-481F-AEEF-1008809A1C8F}"/>
-    <hyperlink ref="C5" r:id="rId13" xr:uid="{EB045B52-E563-41DD-B21B-56FE650FC4E8}"/>
-    <hyperlink ref="D5" r:id="rId14" xr:uid="{0472A11E-E6F2-4BA8-99C9-408E71E9B00D}"/>
-    <hyperlink ref="E5" r:id="rId15" xr:uid="{894D8CE1-A466-412C-B0FC-280C033B8424}"/>
-    <hyperlink ref="B5" r:id="rId16" xr:uid="{0C20EFCD-AD9C-48D6-8730-A6BFF7C17006}"/>
+    <hyperlink ref="C3" r:id="rId4" xr:uid="{548807EE-69C0-4A4D-8A04-AF2D97456A13}"/>
+    <hyperlink ref="D3" r:id="rId5" xr:uid="{5ECCA65F-D672-4C9C-8475-481CB035711B}"/>
+    <hyperlink ref="E3" r:id="rId6" xr:uid="{9CDE25A8-7826-4B6A-9CD2-DA248C33C664}"/>
+    <hyperlink ref="C4" r:id="rId7" xr:uid="{4834B8AE-D2F2-46BB-B1FB-2917FB614179}"/>
+    <hyperlink ref="D4" r:id="rId8" xr:uid="{42D7F317-7486-4C56-8E8B-67291A0DFEBB}"/>
+    <hyperlink ref="E4" r:id="rId9" xr:uid="{3F8C1CEF-9B8C-42CD-8EA8-5A606E73DF96}"/>
+    <hyperlink ref="C5" r:id="rId10" xr:uid="{EB045B52-E563-41DD-B21B-56FE650FC4E8}"/>
+    <hyperlink ref="D5" r:id="rId11" xr:uid="{0472A11E-E6F2-4BA8-99C9-408E71E9B00D}"/>
+    <hyperlink ref="E5" r:id="rId12" xr:uid="{894D8CE1-A466-412C-B0FC-280C033B8424}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId17"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId13"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
patient registration code updated
</commit_message>
<xml_diff>
--- a/src/test/resources/ExcelData/Exceldata.xlsx
+++ b/src/test/resources/ExcelData/Exceldata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Git Projects\SvcProject\src\test\resources\ExcelData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4747744C-6093-433E-892F-46A87B155B6B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C4132A8-2DCF-48D2-82D0-35DB90FB7B74}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" activeTab="5" xr2:uid="{933DE942-FB34-432E-983A-800C465E3B57}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" firstSheet="11" activeTab="11" xr2:uid="{933DE942-FB34-432E-983A-800C465E3B57}"/>
   </bookViews>
   <sheets>
     <sheet name="signupscenarios1" sheetId="5" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="902" uniqueCount="390">
   <si>
     <t>username</t>
   </si>
@@ -808,12 +808,6 @@
     <t>Patient details saved successfully</t>
   </si>
   <si>
-    <t>Rajudeman</t>
-  </si>
-  <si>
-    <t>7589685965</t>
-  </si>
-  <si>
     <t>Patient details updated successfully</t>
   </si>
   <si>
@@ -1198,9 +1192,6 @@
     <t>DeleteReason</t>
   </si>
   <si>
-    <t>8984498911</t>
-  </si>
-  <si>
     <t>account delete</t>
   </si>
   <si>
@@ -1231,9 +1222,6 @@
     <t>ViewPatientSearch</t>
   </si>
   <si>
-    <t>7019619728</t>
-  </si>
-  <si>
     <t>8496345869</t>
   </si>
   <si>
@@ -1241,6 +1229,15 @@
   </si>
   <si>
     <t>Idea@123456</t>
+  </si>
+  <si>
+    <t>7845956958</t>
+  </si>
+  <si>
+    <t>Rajavardhan</t>
+  </si>
+  <si>
+    <t>7845957589</t>
   </si>
 </sst>
 </file>
@@ -1657,7 +1654,7 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>224</v>
@@ -1684,7 +1681,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>223</v>
@@ -1883,85 +1880,85 @@
         <v>213</v>
       </c>
       <c r="L1" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="N1" s="1" t="s">
-        <v>258</v>
-      </c>
       <c r="O1" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="P1" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="P1" s="1" t="s">
-        <v>264</v>
-      </c>
       <c r="Q1" s="1" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="R1" s="1" t="s">
         <v>166</v>
       </c>
       <c r="S1" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="U1" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="U1" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>273</v>
-      </c>
       <c r="W1" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="Y1" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="X1" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>278</v>
-      </c>
       <c r="Z1" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="AB1" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="AD1" s="1" t="s">
-        <v>285</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>286</v>
-      </c>
       <c r="AF1" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="AL1" s="1" t="s">
         <v>293</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>299</v>
-      </c>
-      <c r="AH1" s="1" t="s">
-        <v>300</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>304</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>294</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="2" spans="1:38" x14ac:dyDescent="0.25">
@@ -1972,7 +1969,7 @@
         <v>36</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>21</v>
@@ -1981,7 +1978,7 @@
         <v>22</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>23</v>
@@ -1996,88 +1993,88 @@
         <v>7</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="L2" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="N2" s="1" t="s">
-        <v>259</v>
-      </c>
       <c r="O2" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="P2" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="R2" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="Q2" s="1" t="s">
+      <c r="S2" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="R2" s="1" t="s">
-        <v>268</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>269</v>
-      </c>
       <c r="T2" s="1" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="U2" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="V2" s="1" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="W2" s="1" t="s">
         <v>22</v>
       </c>
       <c r="X2" s="1" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="Y2" s="1" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="Z2" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="AB2" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="AA2" s="1" t="s">
+      <c r="AC2" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="AB2" s="1" t="s">
+      <c r="AD2" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="AC2" s="1" t="s">
+      <c r="AE2" s="1" t="s">
         <v>290</v>
-      </c>
-      <c r="AD2" s="1" t="s">
-        <v>291</v>
-      </c>
-      <c r="AE2" s="1" t="s">
-        <v>292</v>
       </c>
       <c r="AF2" s="1" t="s">
         <v>4</v>
       </c>
       <c r="AG2" s="1" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="AH2" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="AI2" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="AI2" s="1" t="s">
+      <c r="AJ2" s="1" t="s">
         <v>303</v>
       </c>
-      <c r="AJ2" s="1" t="s">
-        <v>305</v>
-      </c>
       <c r="AK2" s="1" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="AL2" s="1" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
   </sheetData>
@@ -2156,7 +2153,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>246</v>
+        <v>388</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>49</v>
@@ -2174,7 +2171,7 @@
         <v>19</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>247</v>
+        <v>389</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>4</v>
@@ -2215,10 +2212,10 @@
         <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>244</v>
@@ -2235,16 +2232,16 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>376</v>
+        <v>387</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
     </row>
   </sheetData>
@@ -2273,10 +2270,10 @@
         <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>244</v>
@@ -2293,16 +2290,16 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
     </row>
   </sheetData>
@@ -2339,7 +2336,7 @@
         <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>39</v>
@@ -2383,10 +2380,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>49</v>
@@ -2403,8 +2400,8 @@
       <c r="I2" t="s">
         <v>19</v>
       </c>
-      <c r="J2">
-        <v>7585469852</v>
+      <c r="J2" s="1" t="s">
+        <v>387</v>
       </c>
       <c r="K2">
         <v>789123</v>
@@ -2416,7 +2413,7 @@
         <v>7</v>
       </c>
       <c r="N2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -2442,7 +2439,7 @@
         <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -2683,7 +2680,7 @@
         <v>7</v>
       </c>
       <c r="W2" s="1" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
   </sheetData>
@@ -2788,7 +2785,7 @@
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>4</v>
@@ -2800,13 +2797,13 @@
         <v>19</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>4</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>76</v>
@@ -2854,7 +2851,7 @@
         <v>7</v>
       </c>
       <c r="W2" s="1" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
   </sheetData>
@@ -3136,7 +3133,7 @@
         <v>7</v>
       </c>
       <c r="W2" s="1" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
   </sheetData>
@@ -3221,7 +3218,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>130</v>
@@ -3254,7 +3251,7 @@
         <v>7</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
   </sheetData>
@@ -3326,7 +3323,7 @@
         <v>7</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -3352,7 +3349,7 @@
         <v>7</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
   </sheetData>
@@ -3426,7 +3423,7 @@
         <v>151</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>23</v>
@@ -3438,7 +3435,7 @@
         <v>7</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
   </sheetData>
@@ -3511,7 +3508,7 @@
         <v>151</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>23</v>
@@ -3523,7 +3520,7 @@
         <v>7</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -3534,16 +3531,16 @@
         <v>4</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>151</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>23</v>
@@ -3555,7 +3552,7 @@
         <v>7</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
   </sheetData>
@@ -3689,7 +3686,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>171</v>
@@ -3719,7 +3716,7 @@
         <v>7</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
   </sheetData>
@@ -3794,7 +3791,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>171</v>
@@ -3824,7 +3821,7 @@
         <v>7</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
   </sheetData>
@@ -3895,7 +3892,7 @@
         <v>170</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>183</v>
@@ -3916,7 +3913,7 @@
         <v>7</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
   </sheetData>
@@ -4009,7 +4006,7 @@
         <v>7</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
   </sheetData>
@@ -4162,7 +4159,7 @@
         <v>7</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -4219,7 +4216,7 @@
         <v>7</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
   </sheetData>
@@ -4270,7 +4267,7 @@
         <v>7</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
   </sheetData>
@@ -4321,7 +4318,7 @@
         <v>7</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -4410,10 +4407,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>203</v>
@@ -4487,7 +4484,7 @@
         <v>232</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -4507,7 +4504,7 @@
         <v>235</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
   </sheetData>
@@ -4534,10 +4531,10 @@
         <v>135</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -4548,10 +4545,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
   </sheetData>
@@ -4583,25 +4580,25 @@
         <v>135</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -4612,25 +4609,25 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>112</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>327</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>328</v>
-      </c>
       <c r="I2" s="1" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
   </sheetData>
@@ -4660,13 +4657,13 @@
         <v>135</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>343</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>344</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>345</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>215</v>
@@ -4677,25 +4674,25 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
   </sheetData>
@@ -4726,16 +4723,16 @@
         <v>135</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>351</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>352</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>353</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>215</v>
@@ -4752,22 +4749,22 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>113</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>355</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>357</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
     </row>
   </sheetData>
@@ -4817,7 +4814,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>8</v>
@@ -4855,13 +4852,13 @@
         <v>135</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>26</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>215</v>
@@ -4885,13 +4882,13 @@
         <v>48</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="H2" s="1"/>
     </row>
@@ -4935,13 +4932,13 @@
         <v>121</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>215</v>
@@ -4961,19 +4958,19 @@
         <v>113</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
   </sheetData>
@@ -5002,10 +4999,10 @@
         <v>135</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>215</v>
@@ -5022,16 +5019,16 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
   </sheetData>
@@ -5060,10 +5057,10 @@
         <v>135</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>215</v>
@@ -5080,16 +5077,16 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
   </sheetData>
@@ -5119,13 +5116,13 @@
         <v>135</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>215</v>
@@ -5142,19 +5139,19 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
   </sheetData>
@@ -5317,10 +5314,10 @@
         <v>36</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>7</v>

</xml_diff>